<commit_message>
feat(riscos): refinamento metodologico UGERC, tela de riscos mapeados e impressao A4
- Implementa catalogo com 11 categorias de risco e sintese de correlacao evento-causa-consequencia
- Adiciona analise de controles internos da Tabela 3 da UGERC (5 niveis com FNC fixo)
- Atualiza seletores de probabilidade e impacto com descricoes normativas e gradiente suave
- Implementa busca combinada por texto e sigla na selecao de Unidades Organizacionais
- Adiciona regra de dependencia sequencial estrita entre as 5 etapas do mapeamento
- Permite salvar rascunho sem redirecionamento de tela
- Cria tela exclusiva de Riscos Mapeados (/riscos/mapeados) com filtros e RBAC restritivo
- Implementa impressao e exportacao da ficha completa em layout A4 multi-paginas sem casca do sistema
- Atualiza e sincroniza especificacoes e mudancas do OpenSpec
</commit_message>
<xml_diff>
--- a/docs/referencias/processos_ebserh/macroprocessos_processos_hospital_tipo_II_Ebserh.xlsx
+++ b/docs/referencias/processos_ebserh/macroprocessos_processos_hospital_tipo_II_Ebserh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ebserhnet-my.sharepoint.com/personal/tassio_silva_ebserh_gov_br/Documents/HC_DEV/Sistema de Gestão de Riscos/docs/referencias/processos_ebserh/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64A70145-67B2-4E25-8CDB-7E52F63879C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{64A70145-67B2-4E25-8CDB-7E52F63879C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F837A24-DE36-4005-B412-5B9FAC606542}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1269,6 +1269,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1277,9 +1280,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1300,7 +1300,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DetalhamentoProcessos" displayName="DetalhamentoProcessos" ref="A1:E246" totalsRowShown="0">
-  <autoFilter ref="A1:E246" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
+  <autoFilter ref="A1:E246" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Hospital Tipo II &gt; Superintendência &gt; SEGOV/Unidade de Planejamento, Gestão de Riscos e Controles Internos"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Área de gestão"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Caminho organizacional no documento"/>
@@ -1547,7 +1553,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" hidden="1">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1564,7 +1570,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" hidden="1">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1581,7 +1587,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" hidden="1">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -1598,7 +1604,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" hidden="1">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -1615,7 +1621,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" hidden="1">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -1632,7 +1638,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" hidden="1">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -1649,7 +1655,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" hidden="1">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
@@ -1666,7 +1672,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="28.5">
+    <row r="9" spans="1:5" ht="28.5" hidden="1">
       <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
@@ -1683,7 +1689,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="28.5">
+    <row r="10" spans="1:5" ht="28.5" hidden="1">
       <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
@@ -1700,7 +1706,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="28.5">
+    <row r="11" spans="1:5" ht="28.5" hidden="1">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -1717,7 +1723,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="28.5">
+    <row r="12" spans="1:5" ht="28.5" hidden="1">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1734,7 +1740,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="28.5">
+    <row r="13" spans="1:5" ht="28.5" hidden="1">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -1751,7 +1757,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="28.5">
+    <row r="14" spans="1:5" ht="28.5" hidden="1">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
@@ -1768,7 +1774,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="28.5">
+    <row r="15" spans="1:5" ht="28.5" hidden="1">
       <c r="A15" s="2" t="s">
         <v>19</v>
       </c>
@@ -1785,7 +1791,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="28.5">
+    <row r="16" spans="1:5" ht="28.5" hidden="1">
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
@@ -1802,7 +1808,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" hidden="1">
       <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
@@ -1819,7 +1825,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" hidden="1">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -2193,7 +2199,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="28.5">
+    <row r="40" spans="1:5" ht="28.5" hidden="1">
       <c r="A40" s="2" t="s">
         <v>19</v>
       </c>
@@ -2210,7 +2216,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="28.5">
+    <row r="41" spans="1:5" ht="28.5" hidden="1">
       <c r="A41" s="2" t="s">
         <v>19</v>
       </c>
@@ -2227,7 +2233,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="28.5">
+    <row r="42" spans="1:5" ht="28.5" hidden="1">
       <c r="A42" s="2" t="s">
         <v>19</v>
       </c>
@@ -2244,7 +2250,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="28.5">
+    <row r="43" spans="1:5" ht="28.5" hidden="1">
       <c r="A43" s="2" t="s">
         <v>19</v>
       </c>
@@ -2261,7 +2267,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="28.5">
+    <row r="44" spans="1:5" ht="28.5" hidden="1">
       <c r="A44" s="2" t="s">
         <v>19</v>
       </c>
@@ -2278,7 +2284,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="28.5">
+    <row r="45" spans="1:5" ht="28.5" hidden="1">
       <c r="A45" s="2" t="s">
         <v>19</v>
       </c>
@@ -2295,7 +2301,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="28.5">
+    <row r="46" spans="1:5" ht="28.5" hidden="1">
       <c r="A46" s="2" t="s">
         <v>19</v>
       </c>
@@ -2312,7 +2318,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="28.5">
+    <row r="47" spans="1:5" ht="28.5" hidden="1">
       <c r="A47" s="2" t="s">
         <v>19</v>
       </c>
@@ -2329,7 +2335,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="28.5">
+    <row r="48" spans="1:5" ht="28.5" hidden="1">
       <c r="A48" s="2" t="s">
         <v>19</v>
       </c>
@@ -2346,7 +2352,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="28.5">
+    <row r="49" spans="1:5" ht="28.5" hidden="1">
       <c r="A49" s="2" t="s">
         <v>19</v>
       </c>
@@ -2363,7 +2369,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="28.5">
+    <row r="50" spans="1:5" ht="28.5" hidden="1">
       <c r="A50" s="2" t="s">
         <v>19</v>
       </c>
@@ -2380,7 +2386,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="28.5">
+    <row r="51" spans="1:5" ht="28.5" hidden="1">
       <c r="A51" s="2" t="s">
         <v>19</v>
       </c>
@@ -2397,7 +2403,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="28.5">
+    <row r="52" spans="1:5" ht="28.5" hidden="1">
       <c r="A52" s="2" t="s">
         <v>19</v>
       </c>
@@ -2414,7 +2420,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="28.5">
+    <row r="53" spans="1:5" ht="28.5" hidden="1">
       <c r="A53" s="2" t="s">
         <v>19</v>
       </c>
@@ -2431,7 +2437,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="28.5">
+    <row r="54" spans="1:5" ht="28.5" hidden="1">
       <c r="A54" s="2" t="s">
         <v>19</v>
       </c>
@@ -2448,7 +2454,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="28.5">
+    <row r="55" spans="1:5" ht="28.5" hidden="1">
       <c r="A55" s="2" t="s">
         <v>19</v>
       </c>
@@ -2465,7 +2471,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="28.5">
+    <row r="56" spans="1:5" ht="28.5" hidden="1">
       <c r="A56" s="2" t="s">
         <v>19</v>
       </c>
@@ -2482,7 +2488,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="28.5">
+    <row r="57" spans="1:5" ht="28.5" hidden="1">
       <c r="A57" s="2" t="s">
         <v>19</v>
       </c>
@@ -2499,7 +2505,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="28.5">
+    <row r="58" spans="1:5" ht="28.5" hidden="1">
       <c r="A58" s="2" t="s">
         <v>19</v>
       </c>
@@ -2516,7 +2522,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" hidden="1">
       <c r="A59" s="2" t="s">
         <v>19</v>
       </c>
@@ -2533,7 +2539,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" hidden="1">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
@@ -2550,7 +2556,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" hidden="1">
       <c r="A61" s="2" t="s">
         <v>19</v>
       </c>
@@ -2567,7 +2573,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" hidden="1">
       <c r="A62" s="2" t="s">
         <v>19</v>
       </c>
@@ -2584,7 +2590,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" hidden="1">
       <c r="A63" s="2" t="s">
         <v>19</v>
       </c>
@@ -2601,7 +2607,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" hidden="1">
       <c r="A64" s="2" t="s">
         <v>19</v>
       </c>
@@ -2618,7 +2624,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" hidden="1">
       <c r="A65" s="2" t="s">
         <v>19</v>
       </c>
@@ -2635,7 +2641,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:5" hidden="1">
       <c r="A66" s="2" t="s">
         <v>19</v>
       </c>
@@ -2652,7 +2658,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:5" hidden="1">
       <c r="A67" s="2" t="s">
         <v>19</v>
       </c>
@@ -2669,7 +2675,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:5" hidden="1">
       <c r="A68" s="2" t="s">
         <v>19</v>
       </c>
@@ -2686,7 +2692,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" hidden="1">
       <c r="A69" s="2" t="s">
         <v>19</v>
       </c>
@@ -2703,7 +2709,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:5" hidden="1">
       <c r="A70" s="2" t="s">
         <v>19</v>
       </c>
@@ -2720,7 +2726,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" spans="1:5" hidden="1">
       <c r="A71" s="2" t="s">
         <v>19</v>
       </c>
@@ -2737,7 +2743,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="28.5">
+    <row r="72" spans="1:5" ht="28.5" hidden="1">
       <c r="A72" s="2" t="s">
         <v>19</v>
       </c>
@@ -2754,7 +2760,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" spans="1:5" hidden="1">
       <c r="A73" s="2" t="s">
         <v>19</v>
       </c>
@@ -2771,7 +2777,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" spans="1:5" hidden="1">
       <c r="A74" s="2" t="s">
         <v>19</v>
       </c>
@@ -2788,7 +2794,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="28.5">
+    <row r="75" spans="1:5" ht="28.5" hidden="1">
       <c r="A75" s="2" t="s">
         <v>19</v>
       </c>
@@ -2805,7 +2811,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="76" spans="1:5" ht="28.5">
+    <row r="76" spans="1:5" ht="28.5" hidden="1">
       <c r="A76" s="2" t="s">
         <v>19</v>
       </c>
@@ -2822,7 +2828,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="77" spans="1:5" ht="28.5">
+    <row r="77" spans="1:5" ht="28.5" hidden="1">
       <c r="A77" s="2" t="s">
         <v>19</v>
       </c>
@@ -2839,7 +2845,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="78" spans="1:5" ht="28.5">
+    <row r="78" spans="1:5" ht="28.5" hidden="1">
       <c r="A78" s="2" t="s">
         <v>19</v>
       </c>
@@ -2856,7 +2862,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="79" spans="1:5" ht="28.5">
+    <row r="79" spans="1:5" ht="28.5" hidden="1">
       <c r="A79" s="2" t="s">
         <v>19</v>
       </c>
@@ -2873,7 +2879,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="80" spans="1:5" ht="28.5">
+    <row r="80" spans="1:5" ht="28.5" hidden="1">
       <c r="A80" s="2" t="s">
         <v>19</v>
       </c>
@@ -2890,7 +2896,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="81" spans="1:5" ht="28.5">
+    <row r="81" spans="1:5" ht="28.5" hidden="1">
       <c r="A81" s="2" t="s">
         <v>19</v>
       </c>
@@ -2907,7 +2913,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:5" hidden="1">
       <c r="A82" s="2" t="s">
         <v>19</v>
       </c>
@@ -2924,7 +2930,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:5" hidden="1">
       <c r="A83" s="2" t="s">
         <v>19</v>
       </c>
@@ -2941,7 +2947,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="84" spans="1:5">
+    <row r="84" spans="1:5" hidden="1">
       <c r="A84" s="2" t="s">
         <v>19</v>
       </c>
@@ -2958,7 +2964,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" spans="1:5" hidden="1">
       <c r="A85" s="2" t="s">
         <v>19</v>
       </c>
@@ -2975,7 +2981,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="86" spans="1:5">
+    <row r="86" spans="1:5" hidden="1">
       <c r="A86" s="2" t="s">
         <v>19</v>
       </c>
@@ -2992,7 +2998,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:5" hidden="1">
       <c r="A87" s="2" t="s">
         <v>19</v>
       </c>
@@ -3009,7 +3015,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="88" spans="1:5">
+    <row r="88" spans="1:5" hidden="1">
       <c r="A88" s="2" t="s">
         <v>19</v>
       </c>
@@ -3026,7 +3032,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="89" spans="1:5">
+    <row r="89" spans="1:5" hidden="1">
       <c r="A89" s="2" t="s">
         <v>19</v>
       </c>
@@ -3043,7 +3049,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" spans="1:5" hidden="1">
       <c r="A90" s="2" t="s">
         <v>19</v>
       </c>
@@ -3060,7 +3066,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="91" spans="1:5">
+    <row r="91" spans="1:5" hidden="1">
       <c r="A91" s="2" t="s">
         <v>19</v>
       </c>
@@ -3077,7 +3083,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" spans="1:5" hidden="1">
       <c r="A92" s="2" t="s">
         <v>19</v>
       </c>
@@ -3094,7 +3100,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="28.5">
+    <row r="93" spans="1:5" ht="28.5" hidden="1">
       <c r="A93" s="2" t="s">
         <v>142</v>
       </c>
@@ -3111,7 +3117,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" spans="1:5" hidden="1">
       <c r="A94" s="2" t="s">
         <v>142</v>
       </c>
@@ -3128,7 +3134,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:5" hidden="1">
       <c r="A95" s="2" t="s">
         <v>142</v>
       </c>
@@ -3145,7 +3151,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="96" spans="1:5">
+    <row r="96" spans="1:5" hidden="1">
       <c r="A96" s="2" t="s">
         <v>142</v>
       </c>
@@ -3162,7 +3168,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="97" spans="1:5">
+    <row r="97" spans="1:5" hidden="1">
       <c r="A97" s="2" t="s">
         <v>142</v>
       </c>
@@ -3179,7 +3185,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="98" spans="1:5">
+    <row r="98" spans="1:5" hidden="1">
       <c r="A98" s="2" t="s">
         <v>142</v>
       </c>
@@ -3196,7 +3202,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="99" spans="1:5">
+    <row r="99" spans="1:5" hidden="1">
       <c r="A99" s="2" t="s">
         <v>142</v>
       </c>
@@ -3213,7 +3219,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="100" spans="1:5">
+    <row r="100" spans="1:5" hidden="1">
       <c r="A100" s="2" t="s">
         <v>142</v>
       </c>
@@ -3230,7 +3236,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="101" spans="1:5">
+    <row r="101" spans="1:5" hidden="1">
       <c r="A101" s="2" t="s">
         <v>142</v>
       </c>
@@ -3247,7 +3253,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" spans="1:5" hidden="1">
       <c r="A102" s="2" t="s">
         <v>142</v>
       </c>
@@ -3264,7 +3270,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" spans="1:5" hidden="1">
       <c r="A103" s="2" t="s">
         <v>142</v>
       </c>
@@ -3281,7 +3287,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" spans="1:5" hidden="1">
       <c r="A104" s="2" t="s">
         <v>142</v>
       </c>
@@ -3298,7 +3304,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" spans="1:5" hidden="1">
       <c r="A105" s="2" t="s">
         <v>142</v>
       </c>
@@ -3315,7 +3321,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="106" spans="1:5">
+    <row r="106" spans="1:5" hidden="1">
       <c r="A106" s="2" t="s">
         <v>142</v>
       </c>
@@ -3332,7 +3338,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="107" spans="1:5">
+    <row r="107" spans="1:5" hidden="1">
       <c r="A107" s="2" t="s">
         <v>142</v>
       </c>
@@ -3349,7 +3355,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="108" spans="1:5">
+    <row r="108" spans="1:5" hidden="1">
       <c r="A108" s="2" t="s">
         <v>142</v>
       </c>
@@ -3366,7 +3372,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="109" spans="1:5">
+    <row r="109" spans="1:5" hidden="1">
       <c r="A109" s="2" t="s">
         <v>142</v>
       </c>
@@ -3383,7 +3389,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="110" spans="1:5" ht="28.5">
+    <row r="110" spans="1:5" ht="28.5" hidden="1">
       <c r="A110" s="2" t="s">
         <v>142</v>
       </c>
@@ -3400,7 +3406,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="111" spans="1:5" ht="28.5">
+    <row r="111" spans="1:5" ht="28.5" hidden="1">
       <c r="A111" s="2" t="s">
         <v>142</v>
       </c>
@@ -3417,7 +3423,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="112" spans="1:5" ht="28.5">
+    <row r="112" spans="1:5" ht="28.5" hidden="1">
       <c r="A112" s="2" t="s">
         <v>142</v>
       </c>
@@ -3434,7 +3440,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="113" spans="1:5" ht="28.5">
+    <row r="113" spans="1:5" ht="28.5" hidden="1">
       <c r="A113" s="2" t="s">
         <v>142</v>
       </c>
@@ -3451,7 +3457,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="114" spans="1:5" ht="28.5">
+    <row r="114" spans="1:5" ht="28.5" hidden="1">
       <c r="A114" s="2" t="s">
         <v>142</v>
       </c>
@@ -3468,7 +3474,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="115" spans="1:5">
+    <row r="115" spans="1:5" hidden="1">
       <c r="A115" s="2" t="s">
         <v>142</v>
       </c>
@@ -3485,7 +3491,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="116" spans="1:5">
+    <row r="116" spans="1:5" hidden="1">
       <c r="A116" s="2" t="s">
         <v>142</v>
       </c>
@@ -3502,7 +3508,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="117" spans="1:5">
+    <row r="117" spans="1:5" hidden="1">
       <c r="A117" s="2" t="s">
         <v>142</v>
       </c>
@@ -3519,7 +3525,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="118" spans="1:5">
+    <row r="118" spans="1:5" hidden="1">
       <c r="A118" s="2" t="s">
         <v>142</v>
       </c>
@@ -3536,7 +3542,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="119" spans="1:5">
+    <row r="119" spans="1:5" hidden="1">
       <c r="A119" s="2" t="s">
         <v>142</v>
       </c>
@@ -3553,7 +3559,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="120" spans="1:5">
+    <row r="120" spans="1:5" hidden="1">
       <c r="A120" s="2" t="s">
         <v>142</v>
       </c>
@@ -3570,7 +3576,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="121" spans="1:5">
+    <row r="121" spans="1:5" hidden="1">
       <c r="A121" s="2" t="s">
         <v>182</v>
       </c>
@@ -3587,7 +3593,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="122" spans="1:5">
+    <row r="122" spans="1:5" hidden="1">
       <c r="A122" s="2" t="s">
         <v>182</v>
       </c>
@@ -3604,7 +3610,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="123" spans="1:5">
+    <row r="123" spans="1:5" hidden="1">
       <c r="A123" s="2" t="s">
         <v>182</v>
       </c>
@@ -3621,7 +3627,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="124" spans="1:5">
+    <row r="124" spans="1:5" hidden="1">
       <c r="A124" s="2" t="s">
         <v>182</v>
       </c>
@@ -3638,7 +3644,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="125" spans="1:5">
+    <row r="125" spans="1:5" hidden="1">
       <c r="A125" s="2" t="s">
         <v>182</v>
       </c>
@@ -3655,7 +3661,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="126" spans="1:5">
+    <row r="126" spans="1:5" hidden="1">
       <c r="A126" s="2" t="s">
         <v>182</v>
       </c>
@@ -3672,7 +3678,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="127" spans="1:5">
+    <row r="127" spans="1:5" hidden="1">
       <c r="A127" s="2" t="s">
         <v>182</v>
       </c>
@@ -3689,7 +3695,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="128" spans="1:5">
+    <row r="128" spans="1:5" hidden="1">
       <c r="A128" s="2" t="s">
         <v>182</v>
       </c>
@@ -3706,7 +3712,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="129" spans="1:5">
+    <row r="129" spans="1:5" hidden="1">
       <c r="A129" s="2" t="s">
         <v>182</v>
       </c>
@@ -3723,7 +3729,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="130" spans="1:5">
+    <row r="130" spans="1:5" hidden="1">
       <c r="A130" s="2" t="s">
         <v>182</v>
       </c>
@@ -3740,7 +3746,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="131" spans="1:5">
+    <row r="131" spans="1:5" hidden="1">
       <c r="A131" s="2" t="s">
         <v>182</v>
       </c>
@@ -3757,7 +3763,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="132" spans="1:5">
+    <row r="132" spans="1:5" hidden="1">
       <c r="A132" s="2" t="s">
         <v>182</v>
       </c>
@@ -3774,7 +3780,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="133" spans="1:5">
+    <row r="133" spans="1:5" hidden="1">
       <c r="A133" s="2" t="s">
         <v>182</v>
       </c>
@@ -3791,7 +3797,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="134" spans="1:5">
+    <row r="134" spans="1:5" hidden="1">
       <c r="A134" s="2" t="s">
         <v>182</v>
       </c>
@@ -3808,7 +3814,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="135" spans="1:5">
+    <row r="135" spans="1:5" hidden="1">
       <c r="A135" s="2" t="s">
         <v>182</v>
       </c>
@@ -3825,7 +3831,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="136" spans="1:5">
+    <row r="136" spans="1:5" hidden="1">
       <c r="A136" s="2" t="s">
         <v>182</v>
       </c>
@@ -3842,7 +3848,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="137" spans="1:5">
+    <row r="137" spans="1:5" hidden="1">
       <c r="A137" s="2" t="s">
         <v>182</v>
       </c>
@@ -3859,7 +3865,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="138" spans="1:5">
+    <row r="138" spans="1:5" hidden="1">
       <c r="A138" s="2" t="s">
         <v>182</v>
       </c>
@@ -3876,7 +3882,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="139" spans="1:5">
+    <row r="139" spans="1:5" hidden="1">
       <c r="A139" s="2" t="s">
         <v>182</v>
       </c>
@@ -3893,7 +3899,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="140" spans="1:5">
+    <row r="140" spans="1:5" hidden="1">
       <c r="A140" s="2" t="s">
         <v>182</v>
       </c>
@@ -3910,7 +3916,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="141" spans="1:5">
+    <row r="141" spans="1:5" hidden="1">
       <c r="A141" s="2" t="s">
         <v>182</v>
       </c>
@@ -3927,7 +3933,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="142" spans="1:5">
+    <row r="142" spans="1:5" hidden="1">
       <c r="A142" s="2" t="s">
         <v>182</v>
       </c>
@@ -3944,7 +3950,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="143" spans="1:5">
+    <row r="143" spans="1:5" hidden="1">
       <c r="A143" s="2" t="s">
         <v>182</v>
       </c>
@@ -3961,7 +3967,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="144" spans="1:5">
+    <row r="144" spans="1:5" hidden="1">
       <c r="A144" s="2" t="s">
         <v>182</v>
       </c>
@@ -3978,7 +3984,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="145" spans="1:5">
+    <row r="145" spans="1:5" hidden="1">
       <c r="A145" s="2" t="s">
         <v>182</v>
       </c>
@@ -3995,7 +4001,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="146" spans="1:5">
+    <row r="146" spans="1:5" hidden="1">
       <c r="A146" s="2" t="s">
         <v>182</v>
       </c>
@@ -4012,7 +4018,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="147" spans="1:5">
+    <row r="147" spans="1:5" hidden="1">
       <c r="A147" s="2" t="s">
         <v>182</v>
       </c>
@@ -4029,7 +4035,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="148" spans="1:5">
+    <row r="148" spans="1:5" hidden="1">
       <c r="A148" s="2" t="s">
         <v>182</v>
       </c>
@@ -4046,7 +4052,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="149" spans="1:5">
+    <row r="149" spans="1:5" hidden="1">
       <c r="A149" s="2" t="s">
         <v>182</v>
       </c>
@@ -4063,7 +4069,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="150" spans="1:5">
+    <row r="150" spans="1:5" hidden="1">
       <c r="A150" s="2" t="s">
         <v>182</v>
       </c>
@@ -4080,7 +4086,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="151" spans="1:5">
+    <row r="151" spans="1:5" hidden="1">
       <c r="A151" s="2" t="s">
         <v>182</v>
       </c>
@@ -4097,7 +4103,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="152" spans="1:5">
+    <row r="152" spans="1:5" hidden="1">
       <c r="A152" s="2" t="s">
         <v>182</v>
       </c>
@@ -4114,7 +4120,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="153" spans="1:5">
+    <row r="153" spans="1:5" hidden="1">
       <c r="A153" s="2" t="s">
         <v>182</v>
       </c>
@@ -4131,7 +4137,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="154" spans="1:5">
+    <row r="154" spans="1:5" hidden="1">
       <c r="A154" s="2" t="s">
         <v>182</v>
       </c>
@@ -4148,7 +4154,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="155" spans="1:5">
+    <row r="155" spans="1:5" hidden="1">
       <c r="A155" s="2" t="s">
         <v>182</v>
       </c>
@@ -4165,7 +4171,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="156" spans="1:5">
+    <row r="156" spans="1:5" hidden="1">
       <c r="A156" s="2" t="s">
         <v>182</v>
       </c>
@@ -4182,7 +4188,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="157" spans="1:5">
+    <row r="157" spans="1:5" hidden="1">
       <c r="A157" s="2" t="s">
         <v>182</v>
       </c>
@@ -4199,7 +4205,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="158" spans="1:5">
+    <row r="158" spans="1:5" hidden="1">
       <c r="A158" s="2" t="s">
         <v>182</v>
       </c>
@@ -4216,7 +4222,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="159" spans="1:5">
+    <row r="159" spans="1:5" hidden="1">
       <c r="A159" s="2" t="s">
         <v>182</v>
       </c>
@@ -4233,7 +4239,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="160" spans="1:5">
+    <row r="160" spans="1:5" hidden="1">
       <c r="A160" s="2" t="s">
         <v>182</v>
       </c>
@@ -4250,7 +4256,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="161" spans="1:5">
+    <row r="161" spans="1:5" hidden="1">
       <c r="A161" s="2" t="s">
         <v>182</v>
       </c>
@@ -4267,7 +4273,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="162" spans="1:5">
+    <row r="162" spans="1:5" hidden="1">
       <c r="A162" s="2" t="s">
         <v>182</v>
       </c>
@@ -4284,7 +4290,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="163" spans="1:5" ht="28.5">
+    <row r="163" spans="1:5" ht="28.5" hidden="1">
       <c r="A163" s="2" t="s">
         <v>182</v>
       </c>
@@ -4301,7 +4307,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="164" spans="1:5" ht="28.5">
+    <row r="164" spans="1:5" ht="28.5" hidden="1">
       <c r="A164" s="2" t="s">
         <v>182</v>
       </c>
@@ -4318,7 +4324,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="165" spans="1:5">
+    <row r="165" spans="1:5" hidden="1">
       <c r="A165" s="2" t="s">
         <v>182</v>
       </c>
@@ -4335,7 +4341,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="166" spans="1:5">
+    <row r="166" spans="1:5" hidden="1">
       <c r="A166" s="2" t="s">
         <v>182</v>
       </c>
@@ -4352,7 +4358,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="167" spans="1:5">
+    <row r="167" spans="1:5" hidden="1">
       <c r="A167" s="2" t="s">
         <v>182</v>
       </c>
@@ -4369,7 +4375,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="168" spans="1:5">
+    <row r="168" spans="1:5" hidden="1">
       <c r="A168" s="2" t="s">
         <v>182</v>
       </c>
@@ -4386,7 +4392,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="169" spans="1:5">
+    <row r="169" spans="1:5" hidden="1">
       <c r="A169" s="2" t="s">
         <v>182</v>
       </c>
@@ -4403,7 +4409,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="170" spans="1:5">
+    <row r="170" spans="1:5" hidden="1">
       <c r="A170" s="2" t="s">
         <v>182</v>
       </c>
@@ -4420,7 +4426,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="171" spans="1:5">
+    <row r="171" spans="1:5" hidden="1">
       <c r="A171" s="2" t="s">
         <v>182</v>
       </c>
@@ -4437,7 +4443,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="172" spans="1:5">
+    <row r="172" spans="1:5" hidden="1">
       <c r="A172" s="2" t="s">
         <v>182</v>
       </c>
@@ -4454,7 +4460,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="173" spans="1:5">
+    <row r="173" spans="1:5" hidden="1">
       <c r="A173" s="2" t="s">
         <v>182</v>
       </c>
@@ -4471,7 +4477,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="174" spans="1:5">
+    <row r="174" spans="1:5" hidden="1">
       <c r="A174" s="2" t="s">
         <v>182</v>
       </c>
@@ -4488,7 +4494,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="175" spans="1:5" ht="28.5">
+    <row r="175" spans="1:5" ht="28.5" hidden="1">
       <c r="A175" s="2" t="s">
         <v>182</v>
       </c>
@@ -4505,7 +4511,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="176" spans="1:5" ht="28.5">
+    <row r="176" spans="1:5" ht="28.5" hidden="1">
       <c r="A176" s="2" t="s">
         <v>182</v>
       </c>
@@ -4522,7 +4528,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="177" spans="1:5" ht="28.5">
+    <row r="177" spans="1:5" ht="28.5" hidden="1">
       <c r="A177" s="2" t="s">
         <v>182</v>
       </c>
@@ -4539,7 +4545,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="178" spans="1:5" ht="28.5">
+    <row r="178" spans="1:5" ht="28.5" hidden="1">
       <c r="A178" s="2" t="s">
         <v>182</v>
       </c>
@@ -4556,7 +4562,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="179" spans="1:5">
+    <row r="179" spans="1:5" hidden="1">
       <c r="A179" s="2" t="s">
         <v>182</v>
       </c>
@@ -4573,7 +4579,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="180" spans="1:5">
+    <row r="180" spans="1:5" hidden="1">
       <c r="A180" s="2" t="s">
         <v>182</v>
       </c>
@@ -4590,7 +4596,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="181" spans="1:5">
+    <row r="181" spans="1:5" hidden="1">
       <c r="A181" s="2" t="s">
         <v>182</v>
       </c>
@@ -4607,7 +4613,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="182" spans="1:5">
+    <row r="182" spans="1:5" hidden="1">
       <c r="A182" s="2" t="s">
         <v>182</v>
       </c>
@@ -4624,7 +4630,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="183" spans="1:5">
+    <row r="183" spans="1:5" hidden="1">
       <c r="A183" s="2" t="s">
         <v>182</v>
       </c>
@@ -4641,7 +4647,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="184" spans="1:5">
+    <row r="184" spans="1:5" hidden="1">
       <c r="A184" s="2" t="s">
         <v>182</v>
       </c>
@@ -4658,7 +4664,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="185" spans="1:5">
+    <row r="185" spans="1:5" hidden="1">
       <c r="A185" s="2" t="s">
         <v>182</v>
       </c>
@@ -4675,7 +4681,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="186" spans="1:5">
+    <row r="186" spans="1:5" hidden="1">
       <c r="A186" s="2" t="s">
         <v>182</v>
       </c>
@@ -4692,7 +4698,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="187" spans="1:5">
+    <row r="187" spans="1:5" hidden="1">
       <c r="A187" s="2" t="s">
         <v>182</v>
       </c>
@@ -4709,7 +4715,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="188" spans="1:5">
+    <row r="188" spans="1:5" hidden="1">
       <c r="A188" s="2" t="s">
         <v>182</v>
       </c>
@@ -4726,7 +4732,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="189" spans="1:5">
+    <row r="189" spans="1:5" hidden="1">
       <c r="A189" s="2" t="s">
         <v>182</v>
       </c>
@@ -4743,7 +4749,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="190" spans="1:5">
+    <row r="190" spans="1:5" hidden="1">
       <c r="A190" s="2" t="s">
         <v>182</v>
       </c>
@@ -4760,7 +4766,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="191" spans="1:5">
+    <row r="191" spans="1:5" hidden="1">
       <c r="A191" s="2" t="s">
         <v>182</v>
       </c>
@@ -4777,7 +4783,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="192" spans="1:5">
+    <row r="192" spans="1:5" hidden="1">
       <c r="A192" s="2" t="s">
         <v>182</v>
       </c>
@@ -4794,7 +4800,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="193" spans="1:5">
+    <row r="193" spans="1:5" hidden="1">
       <c r="A193" s="2" t="s">
         <v>182</v>
       </c>
@@ -4811,7 +4817,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="194" spans="1:5">
+    <row r="194" spans="1:5" hidden="1">
       <c r="A194" s="2" t="s">
         <v>182</v>
       </c>
@@ -4828,7 +4834,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="195" spans="1:5">
+    <row r="195" spans="1:5" hidden="1">
       <c r="A195" s="2" t="s">
         <v>182</v>
       </c>
@@ -4845,7 +4851,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="196" spans="1:5">
+    <row r="196" spans="1:5" hidden="1">
       <c r="A196" s="2" t="s">
         <v>182</v>
       </c>
@@ -4862,7 +4868,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="197" spans="1:5">
+    <row r="197" spans="1:5" hidden="1">
       <c r="A197" s="2" t="s">
         <v>182</v>
       </c>
@@ -4879,7 +4885,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="198" spans="1:5">
+    <row r="198" spans="1:5" hidden="1">
       <c r="A198" s="2" t="s">
         <v>182</v>
       </c>
@@ -4896,7 +4902,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="199" spans="1:5">
+    <row r="199" spans="1:5" hidden="1">
       <c r="A199" s="2" t="s">
         <v>182</v>
       </c>
@@ -4913,7 +4919,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="200" spans="1:5">
+    <row r="200" spans="1:5" hidden="1">
       <c r="A200" s="2" t="s">
         <v>182</v>
       </c>
@@ -4930,7 +4936,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="201" spans="1:5">
+    <row r="201" spans="1:5" hidden="1">
       <c r="A201" s="2" t="s">
         <v>182</v>
       </c>
@@ -4947,7 +4953,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="202" spans="1:5">
+    <row r="202" spans="1:5" hidden="1">
       <c r="A202" s="2" t="s">
         <v>182</v>
       </c>
@@ -4964,7 +4970,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="203" spans="1:5">
+    <row r="203" spans="1:5" hidden="1">
       <c r="A203" s="2" t="s">
         <v>182</v>
       </c>
@@ -4981,7 +4987,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="204" spans="1:5">
+    <row r="204" spans="1:5" hidden="1">
       <c r="A204" s="2" t="s">
         <v>182</v>
       </c>
@@ -4998,7 +5004,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="205" spans="1:5" ht="28.5">
+    <row r="205" spans="1:5" ht="28.5" hidden="1">
       <c r="A205" s="2" t="s">
         <v>182</v>
       </c>
@@ -5015,7 +5021,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="206" spans="1:5">
+    <row r="206" spans="1:5" hidden="1">
       <c r="A206" s="2" t="s">
         <v>182</v>
       </c>
@@ -5032,7 +5038,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="207" spans="1:5">
+    <row r="207" spans="1:5" hidden="1">
       <c r="A207" s="2" t="s">
         <v>182</v>
       </c>
@@ -5049,7 +5055,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="208" spans="1:5">
+    <row r="208" spans="1:5" hidden="1">
       <c r="A208" s="2" t="s">
         <v>182</v>
       </c>
@@ -5066,7 +5072,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="209" spans="1:5">
+    <row r="209" spans="1:5" hidden="1">
       <c r="A209" s="2" t="s">
         <v>182</v>
       </c>
@@ -5083,7 +5089,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="210" spans="1:5">
+    <row r="210" spans="1:5" hidden="1">
       <c r="A210" s="2" t="s">
         <v>182</v>
       </c>
@@ -5100,7 +5106,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="211" spans="1:5" ht="28.5">
+    <row r="211" spans="1:5" ht="28.5" hidden="1">
       <c r="A211" s="2" t="s">
         <v>182</v>
       </c>
@@ -5117,7 +5123,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="212" spans="1:5" ht="28.5">
+    <row r="212" spans="1:5" ht="28.5" hidden="1">
       <c r="A212" s="2" t="s">
         <v>182</v>
       </c>
@@ -5134,7 +5140,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="213" spans="1:5" ht="28.5">
+    <row r="213" spans="1:5" ht="28.5" hidden="1">
       <c r="A213" s="2" t="s">
         <v>182</v>
       </c>
@@ -5151,7 +5157,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="214" spans="1:5" ht="28.5">
+    <row r="214" spans="1:5" ht="28.5" hidden="1">
       <c r="A214" s="2" t="s">
         <v>182</v>
       </c>
@@ -5168,7 +5174,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="215" spans="1:5" ht="28.5">
+    <row r="215" spans="1:5" ht="28.5" hidden="1">
       <c r="A215" s="2" t="s">
         <v>182</v>
       </c>
@@ -5185,7 +5191,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="216" spans="1:5" ht="28.5">
+    <row r="216" spans="1:5" ht="28.5" hidden="1">
       <c r="A216" s="2" t="s">
         <v>182</v>
       </c>
@@ -5202,7 +5208,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="217" spans="1:5">
+    <row r="217" spans="1:5" hidden="1">
       <c r="A217" s="2" t="s">
         <v>315</v>
       </c>
@@ -5219,7 +5225,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="218" spans="1:5" ht="28.5">
+    <row r="218" spans="1:5" ht="28.5" hidden="1">
       <c r="A218" s="2" t="s">
         <v>315</v>
       </c>
@@ -5236,7 +5242,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="219" spans="1:5" ht="28.5">
+    <row r="219" spans="1:5" ht="28.5" hidden="1">
       <c r="A219" s="2" t="s">
         <v>315</v>
       </c>
@@ -5253,7 +5259,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="220" spans="1:5" ht="28.5">
+    <row r="220" spans="1:5" ht="28.5" hidden="1">
       <c r="A220" s="2" t="s">
         <v>315</v>
       </c>
@@ -5270,7 +5276,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="221" spans="1:5" ht="28.5">
+    <row r="221" spans="1:5" ht="28.5" hidden="1">
       <c r="A221" s="2" t="s">
         <v>315</v>
       </c>
@@ -5287,7 +5293,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="222" spans="1:5" ht="28.5">
+    <row r="222" spans="1:5" ht="28.5" hidden="1">
       <c r="A222" s="2" t="s">
         <v>315</v>
       </c>
@@ -5304,7 +5310,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="223" spans="1:5" ht="28.5">
+    <row r="223" spans="1:5" ht="28.5" hidden="1">
       <c r="A223" s="2" t="s">
         <v>315</v>
       </c>
@@ -5321,7 +5327,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="224" spans="1:5" ht="28.5">
+    <row r="224" spans="1:5" ht="28.5" hidden="1">
       <c r="A224" s="2" t="s">
         <v>315</v>
       </c>
@@ -5338,7 +5344,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="225" spans="1:5" ht="28.5">
+    <row r="225" spans="1:5" ht="28.5" hidden="1">
       <c r="A225" s="2" t="s">
         <v>315</v>
       </c>
@@ -5355,7 +5361,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="226" spans="1:5" ht="28.5">
+    <row r="226" spans="1:5" ht="28.5" hidden="1">
       <c r="A226" s="2" t="s">
         <v>315</v>
       </c>
@@ -5372,7 +5378,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="227" spans="1:5" ht="28.5">
+    <row r="227" spans="1:5" ht="28.5" hidden="1">
       <c r="A227" s="2" t="s">
         <v>315</v>
       </c>
@@ -5389,7 +5395,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="228" spans="1:5">
+    <row r="228" spans="1:5" hidden="1">
       <c r="A228" s="2" t="s">
         <v>315</v>
       </c>
@@ -5406,7 +5412,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="229" spans="1:5">
+    <row r="229" spans="1:5" hidden="1">
       <c r="A229" s="2" t="s">
         <v>315</v>
       </c>
@@ -5423,7 +5429,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="230" spans="1:5">
+    <row r="230" spans="1:5" hidden="1">
       <c r="A230" s="2" t="s">
         <v>315</v>
       </c>
@@ -5440,7 +5446,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="231" spans="1:5">
+    <row r="231" spans="1:5" hidden="1">
       <c r="A231" s="2" t="s">
         <v>315</v>
       </c>
@@ -5457,7 +5463,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="232" spans="1:5">
+    <row r="232" spans="1:5" hidden="1">
       <c r="A232" s="2" t="s">
         <v>315</v>
       </c>
@@ -5474,7 +5480,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="233" spans="1:5">
+    <row r="233" spans="1:5" hidden="1">
       <c r="A233" s="2" t="s">
         <v>315</v>
       </c>
@@ -5491,7 +5497,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="234" spans="1:5">
+    <row r="234" spans="1:5" hidden="1">
       <c r="A234" s="2" t="s">
         <v>315</v>
       </c>
@@ -5508,7 +5514,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="235" spans="1:5">
+    <row r="235" spans="1:5" hidden="1">
       <c r="A235" s="2" t="s">
         <v>315</v>
       </c>
@@ -5525,7 +5531,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="236" spans="1:5">
+    <row r="236" spans="1:5" hidden="1">
       <c r="A236" s="2" t="s">
         <v>315</v>
       </c>
@@ -5542,7 +5548,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="237" spans="1:5">
+    <row r="237" spans="1:5" hidden="1">
       <c r="A237" s="2" t="s">
         <v>315</v>
       </c>
@@ -5559,7 +5565,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="238" spans="1:5">
+    <row r="238" spans="1:5" hidden="1">
       <c r="A238" s="2" t="s">
         <v>315</v>
       </c>
@@ -5576,7 +5582,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="239" spans="1:5">
+    <row r="239" spans="1:5" hidden="1">
       <c r="A239" s="2" t="s">
         <v>315</v>
       </c>
@@ -5593,7 +5599,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="240" spans="1:5">
+    <row r="240" spans="1:5" hidden="1">
       <c r="A240" s="2" t="s">
         <v>315</v>
       </c>
@@ -5610,7 +5616,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="241" spans="1:5">
+    <row r="241" spans="1:5" hidden="1">
       <c r="A241" s="2" t="s">
         <v>315</v>
       </c>
@@ -5627,7 +5633,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="242" spans="1:5">
+    <row r="242" spans="1:5" hidden="1">
       <c r="A242" s="2" t="s">
         <v>315</v>
       </c>
@@ -5644,7 +5650,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="243" spans="1:5">
+    <row r="243" spans="1:5" hidden="1">
       <c r="A243" s="2" t="s">
         <v>315</v>
       </c>
@@ -5661,7 +5667,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="244" spans="1:5">
+    <row r="244" spans="1:5" hidden="1">
       <c r="A244" s="2" t="s">
         <v>315</v>
       </c>
@@ -5678,7 +5684,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="245" spans="1:5">
+    <row r="245" spans="1:5" hidden="1">
       <c r="A245" s="2" t="s">
         <v>315</v>
       </c>
@@ -5695,7 +5701,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="246" spans="1:5" ht="28.5">
+    <row r="246" spans="1:5" ht="28.5" hidden="1">
       <c r="A246" s="2" t="s">
         <v>315</v>
       </c>
@@ -6327,22 +6333,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>363</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" ht="32.1" customHeight="1">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>364</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
     </row>
     <row r="4" spans="1:5" ht="15">
       <c r="A4" s="4" t="s">
@@ -6479,67 +6485,67 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="26.1" customHeight="1">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="9" t="s">
         <v>373</v>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
     </row>
     <row r="19" spans="1:5" ht="36" customHeight="1">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
     </row>
     <row r="20" spans="1:5" ht="36" customHeight="1">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="6" t="s">
         <v>375</v>
       </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
     </row>
     <row r="21" spans="1:5" ht="36" customHeight="1">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
     </row>
     <row r="22" spans="1:5" ht="36" customHeight="1">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
     </row>
     <row r="23" spans="1:5" ht="36" customHeight="1">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
     </row>
     <row r="24" spans="1:5" ht="36" customHeight="1">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="6" t="s">
         <v>379</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>